<commit_message>
maj de tableau e5
</commit_message>
<xml_diff>
--- a/public/docs/tableau-e5-synthese.xlsx
+++ b/public/docs/tableau-e5-synthese.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$28</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
   <extLst>
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
   <si>
     <t xml:space="preserve">BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
   <si>
-    <t xml:space="preserve">SESSION 2025</t>
+    <t xml:space="preserve">SESSION 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau de synthèse des réalisations professionnelles </t>
@@ -34,7 +34,7 @@
     <t xml:space="preserve">NOM et prénom : SRIKANTHAN Sabiran</t>
   </si>
   <si>
-    <t xml:space="preserve">N° candidat : </t>
+    <t xml:space="preserve">N° candidat : 2541474886 </t>
   </si>
   <si>
     <t xml:space="preserve">Centre de formation : IPSSI PARIS</t>
@@ -49,7 +49,7 @@
     <t xml:space="preserve">▢ SLAM</t>
   </si>
   <si>
-    <t xml:space="preserve">Adresse URL du portfolio : localhost:2368</t>
+    <t xml:space="preserve">Adresse URL du portfolio : https://sabi0407.github.io/s.sabiran/</t>
   </si>
   <si>
     <t xml:space="preserve">Compétences mises en œuvre
@@ -116,64 +116,130 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">Mise en place de mon portfolio</t>
+  </si>
+  <si>
+    <t>15/10/24</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
     <t xml:space="preserve">AP1: Création d’une entreprise fictif et d’une vitrine de site internet pour vendre des services</t>
   </si>
   <si>
-    <t>10/24</t>
+    <t>22/10/24</t>
   </si>
   <si>
     <t>X</t>
   </si>
   <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise en place de Windows server et intégration dans un localdomain</t>
+  </si>
+  <si>
+    <t>13/11/24</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise en place d'un système de ticketing (GLPI)</t>
+  </si>
+  <si>
+    <t>12/02/25</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise en place d’un serveur web avec redirection HTTPS</t>
+  </si>
+  <si>
+    <t>28/03/25</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
     <t xml:space="preserve">AP2: Présentation des avantages de GLPI et de ANSIBLE</t>
   </si>
   <si>
-    <t>04/25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mise en place de mon portfolio </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Veille Technologique </t>
-  </si>
-  <si>
-    <t>05/25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mise en place d'un système de ticketing (GLPI)</t>
-  </si>
-  <si>
-    <t>02/25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mise en place de Windows server et intégration dans un localdomain</t>
-  </si>
-  <si>
-    <t>11/24</t>
-  </si>
-  <si>
-    <t>x</t>
+    <t>02/04/25</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
   <si>
     <t xml:space="preserve">Mise en place d’un loadbalancer</t>
   </si>
   <si>
-    <t xml:space="preserve">Mise en place d’un serveur web avec redirection HTTPS</t>
-  </si>
-  <si>
-    <t>03/25</t>
+    <t>16/04/25</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Veille Technologique</t>
+  </si>
+  <si>
+    <t>12/05/25</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
   <si>
     <t xml:space="preserve">Mise en placce de Zabbix et de ses agents (Windows &amp; Linux)</t>
   </si>
   <si>
-    <t>02/26</t>
+    <t>04/02/26</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
   <si>
     <t xml:space="preserve">Mise en place d'un serveur de sauvegarde Proxmox Backup Server</t>
   </si>
   <si>
-    <t>03/26</t>
+    <t>27/03/26</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
   <si>
     <t xml:space="preserve">Réalisations en milieu professionnel en cours de première année</t>
@@ -182,43 +248,139 @@
     <t xml:space="preserve">Mise en place d’un Serveur Proxmox</t>
   </si>
   <si>
+    <t>08/04/25</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mise en place d’un Portail Captif avec Alcasar</t>
   </si>
   <si>
+    <t>09/04/25</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personnalisation du portail captif ALCASAR</t>
+  </si>
+  <si>
+    <t>10/04/25</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
     <t xml:space="preserve">Création de filtrages DNS</t>
   </si>
   <si>
-    <t xml:space="preserve">Création d’une interface connexion avec AutoIT via API de ALCASAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configuration LAN &amp; WAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sécurisé le navigateur Firefox </t>
+    <t>19/05/25</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sécurisation et configuration du navigateur Firefox et configuration LAN/WAN</t>
+  </si>
+  <si>
+    <t>27/05/25</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
   <si>
     <t xml:space="preserve">Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
-    <t xml:space="preserve">Préparation et configuration de postes informatiques (imprimantes, ordinateurs portable et portable professionnel)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Support informatique niveau 1 aux utilisateurs (Résolution de problème réseau, problème d'impression...)</t>
   </si>
   <si>
-    <t xml:space="preserve">Assurer le bon fonctionnement des outils informatiques (résoudre les panne plus rapidement possible, éviter que le travail soit bloqué trop longtemps)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Participation à la migration des postes vers Entra ID et Intune (Sortie d’Active Directory et migration 100 % cloud via Entra ID / Intune)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Onboarding et accompagnement des utilisateurs ( création des utilisateurs, préparer et configurer son PC, installer les logiciels nécessaires, lui expliquer comment utiliser les outils, </t>
-  </si>
-  <si>
-    <t xml:space="preserve">x </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Développement des compétences en support informatique ( apprendre à mieux dépanner les postes utilisateurs, devenir plus autonome sur les incidents, mieux utiliser les outils, appliquer les procédures .)</t>
+    <t>18/09/25</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résolution de ticket via TIKIT</t>
+  </si>
+  <si>
+    <t>30/09/25</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onboarding et accompagnement des utilisateurs ( création des utilisateurs, préparer et configurer son PC et portable, installer les logiciels nécessaires, lui expliquer comment utiliser les outils,</t>
+  </si>
+  <si>
+    <t>15/10/25</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -228,7 +390,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* \-??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <sz val="10.000000"/>
       <color theme="1"/>
@@ -292,11 +454,6 @@
       <sz val="24.000000"/>
       <name val="Adwaita Mono"/>
     </font>
-    <font>
-      <b/>
-      <sz val="24.000000"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -650,7 +807,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="43">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment vertical="center"/>
@@ -724,18 +881,15 @@
     <xf fontId="10" fillId="0" borderId="22" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf fontId="9" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf fontId="10" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="11" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="8" fillId="0" borderId="22" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="9" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="7" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -744,13 +898,7 @@
     </xf>
     <xf fontId="0" fillId="0" borderId="7" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" quotePrefix="0" pivotButton="0"/>
     <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="7" fillId="0" borderId="22" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf fontId="12" fillId="0" borderId="22" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="13" fillId="0" borderId="22" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
@@ -1182,7 +1330,7 @@
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.859375" defaultRowHeight="12.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" style="1" width="102.421875"/>
-    <col customWidth="1" min="2" max="2" style="1" width="24"/>
+    <col customWidth="1" min="2" max="2" style="1" width="21.421875"/>
     <col customWidth="1" min="3" max="8" style="1" width="18.710000000000001"/>
     <col customWidth="1" min="9" max="43" width="11.43"/>
     <col customWidth="1" min="44" max="16384" style="1" width="10.85"/>
@@ -1315,18 +1463,14 @@
       <c r="B9" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="29" t="s">
-        <v>27</v>
-      </c>
+      <c r="C9" s="29"/>
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
-      <c r="F9" s="29" t="s">
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="H9" s="31"/>
     </row>
     <row r="10" s="21" customFormat="1" ht="39.75" customHeight="1">
       <c r="A10" s="27" t="s">
@@ -1336,555 +1480,504 @@
         <v>29</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D10" s="30"/>
       <c r="E10" s="30"/>
       <c r="F10" s="29" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G10" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="31"/>
+        <v>32</v>
+      </c>
+      <c r="H10" s="32"/>
     </row>
     <row r="11" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A11" s="32" t="s">
-        <v>30</v>
+      <c r="A11" s="33" t="s">
+        <v>33</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="33"/>
+        <v>34</v>
+      </c>
+      <c r="C11" s="29" t="s">
+        <v>35</v>
+      </c>
       <c r="D11" s="30"/>
       <c r="E11" s="30"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="34" t="s">
-        <v>27</v>
-      </c>
+      <c r="F11" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="G11" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" s="31"/>
     </row>
     <row r="12" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A12" s="32" t="s">
-        <v>31</v>
+      <c r="A12" s="33" t="s">
+        <v>38</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="30"/>
+        <v>39</v>
+      </c>
+      <c r="C12" s="29" t="s">
+        <v>40</v>
+      </c>
       <c r="D12" s="30"/>
       <c r="E12" s="30"/>
       <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="34" t="s">
-        <v>27</v>
-      </c>
+      <c r="G12" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" s="31"/>
     </row>
     <row r="13" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A13" s="32" t="s">
-        <v>33</v>
+      <c r="A13" s="33" t="s">
+        <v>42</v>
       </c>
       <c r="B13" s="28" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="D13" s="30"/>
       <c r="E13" s="30"/>
       <c r="F13" s="30"/>
       <c r="G13" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="31"/>
+        <v>45</v>
+      </c>
+      <c r="H13" s="32"/>
     </row>
     <row r="14" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A14" s="35" t="s">
-        <v>35</v>
+      <c r="A14" s="34" t="s">
+        <v>46</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="D14" s="30"/>
       <c r="E14" s="30"/>
       <c r="F14" s="29" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="H14" s="31"/>
+        <v>50</v>
+      </c>
+      <c r="H14" s="32"/>
     </row>
     <row r="15" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A15" s="35" t="s">
-        <v>38</v>
+      <c r="A15" s="34" t="s">
+        <v>51</v>
       </c>
       <c r="B15" s="28" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="D15" s="30"/>
       <c r="E15" s="30"/>
       <c r="F15" s="29" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="G15" s="30"/>
-      <c r="H15" s="31"/>
+      <c r="H15" s="32"/>
     </row>
     <row r="16" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A16" s="35" t="s">
-        <v>39</v>
+      <c r="A16" s="34" t="s">
+        <v>55</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>37</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C16" s="29"/>
       <c r="D16" s="30"/>
       <c r="E16" s="30"/>
       <c r="F16" s="30"/>
-      <c r="G16" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="H16" s="31"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="31" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="17" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A17" s="35" t="s">
-        <v>41</v>
+      <c r="A17" s="34" t="s">
+        <v>58</v>
       </c>
       <c r="B17" s="28" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="D17" s="30"/>
       <c r="E17" s="30"/>
       <c r="F17" s="29" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="H17" s="31"/>
+        <v>62</v>
+      </c>
+      <c r="H17" s="32"/>
     </row>
     <row r="18" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A18" s="35" t="s">
-        <v>43</v>
+      <c r="A18" s="34" t="s">
+        <v>63</v>
       </c>
       <c r="B18" s="28" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="D18" s="30"/>
       <c r="E18" s="30"/>
       <c r="F18" s="29" t="s">
-        <v>37</v>
+        <v>66</v>
       </c>
       <c r="G18" s="30"/>
-      <c r="H18" s="31"/>
+      <c r="H18" s="32"/>
     </row>
     <row r="19" s="21" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A19" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19" s="37"/>
+      <c r="A19" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="B19" s="36"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
-      <c r="H19" s="38"/>
+      <c r="H19" s="37"/>
     </row>
     <row r="20" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A20" s="35" t="s">
-        <v>46</v>
+      <c r="A20" s="34" t="s">
+        <v>68</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>37</v>
+        <v>70</v>
       </c>
       <c r="D20" s="29"/>
       <c r="E20" s="29"/>
       <c r="F20" s="29" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="G20" s="29"/>
-      <c r="H20" s="34" t="s">
-        <v>37</v>
+      <c r="H20" s="31" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="21" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A21" s="35" t="s">
-        <v>47</v>
+      <c r="A21" s="34" t="s">
+        <v>73</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="C21" s="29" t="s">
-        <v>37</v>
+        <v>75</v>
       </c>
       <c r="D21" s="29" t="s">
-        <v>37</v>
+        <v>76</v>
       </c>
       <c r="E21" s="29"/>
       <c r="F21" s="29" t="s">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="G21" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="H21" s="34" t="s">
-        <v>37</v>
+        <v>78</v>
+      </c>
+      <c r="H21" s="31" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="22" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A22" s="35" t="s">
-        <v>48</v>
+      <c r="A22" s="34" t="s">
+        <v>80</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="D22" s="29" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="E22" s="29"/>
       <c r="F22" s="29" t="s">
-        <v>37</v>
+        <v>84</v>
       </c>
       <c r="G22" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="H22" s="34" t="s">
-        <v>37</v>
+        <v>85</v>
+      </c>
+      <c r="H22" s="31" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="23" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A23" s="35" t="s">
-        <v>49</v>
+      <c r="A23" s="34" t="s">
+        <v>87</v>
       </c>
       <c r="B23" s="28" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="29"/>
+        <v>88</v>
+      </c>
+      <c r="C23" s="29" t="s">
+        <v>89</v>
+      </c>
       <c r="D23" s="29" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="E23" s="29"/>
       <c r="F23" s="29" t="s">
-        <v>37</v>
+        <v>91</v>
       </c>
       <c r="G23" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="H23" s="34" t="s">
-        <v>37</v>
+        <v>92</v>
+      </c>
+      <c r="H23" s="31" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="24" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A24" s="35" t="s">
-        <v>50</v>
+      <c r="A24" s="34" t="s">
+        <v>94</v>
       </c>
       <c r="B24" s="28" t="s">
-        <v>29</v>
+        <v>95</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>37</v>
+        <v>96</v>
       </c>
       <c r="D24" s="29" t="s">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E24" s="29"/>
       <c r="F24" s="29" t="s">
-        <v>37</v>
+        <v>98</v>
       </c>
       <c r="G24" s="29"/>
-      <c r="H24" s="34"/>
-    </row>
-    <row r="25" s="21" customFormat="1" ht="39.75" customHeight="1">
+      <c r="H24" s="31" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="25" s="21" customFormat="1" ht="16.5" customHeight="1">
       <c r="A25" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="B25" s="28" t="s">
-        <v>32</v>
-      </c>
-      <c r="C25" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="D25" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="34" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="26" s="21" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A26" s="36" t="s">
-        <v>52</v>
-      </c>
-      <c r="B26" s="37"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="38"/>
+        <v>100</v>
+      </c>
+      <c r="B25" s="36"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="37"/>
+    </row>
+    <row r="26" s="21" customFormat="1" ht="39.75" customHeight="1">
+      <c r="A26" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="C26" s="38"/>
+      <c r="D26" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="E26" s="30"/>
+      <c r="F26" s="30"/>
+      <c r="G26" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="H26" s="32"/>
     </row>
     <row r="27" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A27" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="B27" s="39"/>
-      <c r="C27" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="D27" s="30"/>
+      <c r="A27" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="B27" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29" t="s">
+        <v>107</v>
+      </c>
       <c r="E27" s="30"/>
       <c r="F27" s="30"/>
-      <c r="G27" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H27" s="31"/>
+      <c r="G27" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="H27" s="32"/>
     </row>
     <row r="28" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A28" s="35" t="s">
-        <v>54</v>
-      </c>
-      <c r="B28" s="39"/>
-      <c r="C28" s="30"/>
-      <c r="D28" s="40" t="s">
-        <v>37</v>
+      <c r="A28" s="34" t="s">
+        <v>109</v>
+      </c>
+      <c r="B28" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="C28" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="D28" s="29" t="s">
+        <v>112</v>
       </c>
       <c r="E28" s="30"/>
       <c r="F28" s="30"/>
-      <c r="G28" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="H28" s="31"/>
-    </row>
-    <row r="29" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A29" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="B29" s="39"/>
-      <c r="C29" s="30"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="30"/>
-      <c r="F29" s="30"/>
-      <c r="G29" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="H29" s="31"/>
-    </row>
-    <row r="30" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A30" s="35" t="s">
-        <v>56</v>
-      </c>
-      <c r="B30" s="39"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="E30" s="30"/>
-      <c r="F30" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="G30" s="30"/>
-      <c r="H30" s="31"/>
-    </row>
-    <row r="31" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A31" s="35" t="s">
-        <v>57</v>
-      </c>
-      <c r="B31" s="39"/>
-      <c r="C31" s="41" t="s">
-        <v>58</v>
-      </c>
-      <c r="D31" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="E31" s="30"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="30"/>
-      <c r="H31" s="31"/>
-    </row>
-    <row r="32" s="21" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A32" s="35" t="s">
-        <v>59</v>
-      </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="30"/>
-      <c r="D32" s="30"/>
-      <c r="E32" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="31"/>
-    </row>
-    <row r="33" s="21" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A33" s="42"/>
-      <c r="B33" s="43"/>
-      <c r="C33" s="44"/>
-      <c r="D33" s="44"/>
-      <c r="E33" s="44"/>
-      <c r="F33" s="44"/>
-      <c r="G33" s="44"/>
-      <c r="H33" s="44"/>
+      <c r="G28" s="29" t="s">
+        <v>113</v>
+      </c>
+      <c r="H28" s="32"/>
+    </row>
+    <row r="29" s="21" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A29" s="39"/>
+      <c r="B29" s="40"/>
+      <c r="C29" s="41"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="41"/>
+      <c r="F29" s="41"/>
+      <c r="G29" s="41"/>
+      <c r="H29" s="41"/>
+    </row>
+    <row r="30" ht="12.75" customHeight="1">
+      <c r="B30" s="42"/>
+    </row>
+    <row r="31" ht="12.75" customHeight="1">
+      <c r="B31" s="42"/>
+    </row>
+    <row r="32" ht="12.75" customHeight="1">
+      <c r="B32" s="42"/>
+    </row>
+    <row r="33" ht="12.75" customHeight="1">
+      <c r="B33" s="42"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
-      <c r="B34" s="45"/>
+      <c r="B34" s="42"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
-      <c r="B35" s="45"/>
+      <c r="B35" s="42"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
-      <c r="B36" s="45"/>
+      <c r="B36" s="42"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
-      <c r="B37" s="45"/>
+      <c r="B37" s="42"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
-      <c r="B38" s="45"/>
+      <c r="B38" s="42"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
-      <c r="B39" s="45"/>
+      <c r="B39" s="42"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
-      <c r="B40" s="45"/>
+      <c r="B40" s="42"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
-      <c r="B41" s="45"/>
+      <c r="B41" s="42"/>
     </row>
     <row r="42" ht="12.75" customHeight="1">
-      <c r="B42" s="45"/>
+      <c r="B42" s="42"/>
     </row>
     <row r="43" ht="12.75" customHeight="1">
-      <c r="B43" s="45"/>
+      <c r="B43" s="42"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
-      <c r="B44" s="45"/>
+      <c r="B44" s="42"/>
     </row>
     <row r="45" ht="12.75" customHeight="1">
-      <c r="B45" s="45"/>
+      <c r="B45" s="42"/>
     </row>
     <row r="46" ht="12.75" customHeight="1">
-      <c r="B46" s="45"/>
+      <c r="B46" s="42"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
-      <c r="B47" s="45"/>
+      <c r="B47" s="42"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
-      <c r="B48" s="45"/>
+      <c r="B48" s="42"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
-      <c r="B49" s="45"/>
+      <c r="B49" s="42"/>
     </row>
     <row r="50" ht="12.75" customHeight="1">
-      <c r="B50" s="45"/>
+      <c r="B50" s="42"/>
     </row>
     <row r="51" ht="12.75" customHeight="1">
-      <c r="B51" s="45"/>
+      <c r="B51" s="42"/>
     </row>
     <row r="52" ht="12.75" customHeight="1">
-      <c r="B52" s="45"/>
+      <c r="B52" s="42"/>
     </row>
     <row r="53" ht="12.75" customHeight="1">
-      <c r="B53" s="45"/>
+      <c r="B53" s="42"/>
     </row>
     <row r="54" ht="12.75" customHeight="1">
-      <c r="B54" s="45"/>
+      <c r="B54" s="42"/>
     </row>
     <row r="55" ht="12.75" customHeight="1">
-      <c r="B55" s="45"/>
+      <c r="B55" s="42"/>
     </row>
     <row r="56" ht="12.75" customHeight="1">
-      <c r="B56" s="45"/>
+      <c r="B56" s="42"/>
     </row>
     <row r="57" ht="12.75" customHeight="1">
-      <c r="B57" s="45"/>
+      <c r="B57" s="42"/>
     </row>
     <row r="58" ht="12.75" customHeight="1">
-      <c r="B58" s="45"/>
+      <c r="B58" s="42"/>
     </row>
     <row r="59" ht="12.75" customHeight="1">
-      <c r="B59" s="45"/>
+      <c r="B59" s="42"/>
     </row>
     <row r="60" ht="12.75" customHeight="1">
-      <c r="B60" s="45"/>
+      <c r="B60" s="42"/>
     </row>
     <row r="61" ht="12.75" customHeight="1">
-      <c r="B61" s="45"/>
+      <c r="B61" s="42"/>
     </row>
     <row r="62" ht="12.75" customHeight="1">
-      <c r="B62" s="45"/>
+      <c r="B62" s="42"/>
     </row>
     <row r="63" ht="12.75" customHeight="1">
-      <c r="B63" s="45"/>
+      <c r="B63" s="42"/>
     </row>
     <row r="64" ht="12.75" customHeight="1">
-      <c r="B64" s="45"/>
+      <c r="B64" s="42"/>
     </row>
     <row r="65" ht="12.75" customHeight="1">
-      <c r="B65" s="45"/>
+      <c r="B65" s="42"/>
     </row>
     <row r="66" ht="12.75" customHeight="1">
-      <c r="B66" s="45"/>
+      <c r="B66" s="42"/>
     </row>
     <row r="67" ht="12.75" customHeight="1">
-      <c r="B67" s="45"/>
+      <c r="B67" s="42"/>
     </row>
     <row r="68" ht="12.75" customHeight="1">
-      <c r="B68" s="45"/>
+      <c r="B68" s="42"/>
     </row>
     <row r="69" ht="12.75" customHeight="1">
-      <c r="B69" s="45"/>
+      <c r="B69" s="42"/>
     </row>
     <row r="70" ht="12.75" customHeight="1">
-      <c r="B70" s="45"/>
+      <c r="B70" s="42"/>
     </row>
     <row r="71" ht="12.75" customHeight="1">
-      <c r="B71" s="45"/>
+      <c r="B71" s="42"/>
     </row>
     <row r="72" ht="12.75" customHeight="1">
-      <c r="B72" s="45"/>
+      <c r="B72" s="42"/>
     </row>
     <row r="73" ht="12.75" customHeight="1">
-      <c r="B73" s="45"/>
+      <c r="B73" s="42"/>
     </row>
     <row r="74" ht="12.75" customHeight="1">
-      <c r="B74" s="45"/>
-    </row>
-    <row r="75" ht="12.75" customHeight="1">
-      <c r="B75" s="45"/>
-    </row>
-    <row r="76" ht="12.75" customHeight="1">
-      <c r="B76" s="45"/>
-    </row>
-    <row r="77" ht="12.75" customHeight="1">
-      <c r="B77" s="45"/>
-    </row>
-    <row r="78" ht="12.75" customHeight="1">
-      <c r="B78" s="45"/>
-    </row>
-    <row r="79" ht="12.75" customHeight="1">
-      <c r="B79" s="45"/>
+      <c r="B74" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -1899,11 +1992,11 @@
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A25:H25"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0" horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19652777777777802" right="0.19652777777777802" top="0.19652777777777802" bottom="0.19652777777777802" header="0.51181102362204689" footer="0.51181102362204689"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="44" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>